<commit_message>
Content of assignment 3_mendel_metrics a study of mendelbroat script performance thorugh the use of OpenMP.
</commit_message>
<xml_diff>
--- a/3_assignments/3_mendel_metrics/metrics.xlsx
+++ b/3_assignments/3_mendel_metrics/metrics.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Viccari\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Viccari\Documents\repos\master_udesc_ppgca\course_ppa\3_assignments\3_mendel_metrics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86CE8F1E-61DA-4DD7-A0EA-CB4CDC34BF09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{355DFAE3-294E-4443-8D35-50BFD261C4FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4335" yWindow="1155" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18675" yWindow="0" windowWidth="10230" windowHeight="15585" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="39">
   <si>
     <t>mandelbrot</t>
   </si>
@@ -136,12 +138,22 @@
   </si>
   <si>
     <t>10.5</t>
+  </si>
+  <si>
+    <t># threads</t>
+  </si>
+  <si>
+    <t># chunk</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
+    <numFmt numFmtId="168" formatCode="0.00000"/>
+    <numFmt numFmtId="173" formatCode="#,##0.00000"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -171,7 +183,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -180,14 +192,17 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -493,7 +508,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="4" t="s">
         <v>23</v>
       </c>
     </row>
@@ -508,7 +523,7 @@
         <v>3300</v>
       </c>
       <c r="B3" s="2"/>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="4" t="s">
         <v>33</v>
       </c>
     </row>
@@ -517,7 +532,7 @@
         <v>790</v>
       </c>
       <c r="B4" s="2"/>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="4" t="s">
         <v>34</v>
       </c>
     </row>
@@ -526,7 +541,7 @@
         <v>2400</v>
       </c>
       <c r="B5" s="2"/>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="4" t="s">
         <v>35</v>
       </c>
     </row>
@@ -534,49 +549,49 @@
       <c r="A7" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="F7" s="4" t="s">
+      <c r="E7" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="H7" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="I7" s="4" t="s">
+      <c r="H7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="J7" s="4" t="s">
+      <c r="J7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K7" s="4" t="s">
+      <c r="K7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="L7" s="4" t="s">
+      <c r="L7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M7" s="4" t="s">
+      <c r="M7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="N7" s="4" t="s">
+      <c r="N7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="O7" s="4" t="s">
+      <c r="O7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="P7" s="4" t="s">
+      <c r="P7" s="2" t="s">
         <v>20</v>
       </c>
     </row>
@@ -584,43 +599,43 @@
       <c r="A8" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="5">
+      <c r="B8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="3">
         <v>85942</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="3">
         <v>32054</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="3">
         <v>12567</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="3">
         <v>4332</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="3">
         <v>12443</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="3">
         <v>4348</v>
       </c>
-      <c r="I8" s="5">
+      <c r="I8" s="3">
         <v>8792</v>
       </c>
-      <c r="J8" s="4" t="s">
+      <c r="J8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="3">
         <v>1446</v>
       </c>
-      <c r="L8" s="5">
+      <c r="L8" s="3">
         <v>9988</v>
       </c>
-      <c r="M8" s="5">
+      <c r="M8" s="3">
         <v>3149</v>
       </c>
-      <c r="N8" s="5">
+      <c r="N8" s="3">
         <v>12975</v>
       </c>
       <c r="O8" s="1">
@@ -634,27 +649,26 @@
       <c r="A9" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5">
+      <c r="B9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3">
         <v>12849</v>
       </c>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5">
+      <c r="H9" s="3"/>
+      <c r="I9" s="3">
         <v>8315</v>
       </c>
-      <c r="J9" s="4"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5">
+      <c r="K9" s="3"/>
+      <c r="L9" s="3">
         <v>10355</v>
       </c>
-      <c r="M9" s="5"/>
-      <c r="N9" s="5">
+      <c r="M9" s="3"/>
+      <c r="N9" s="3">
         <v>13429</v>
       </c>
       <c r="O9" s="1"/>
@@ -664,27 +678,26 @@
       <c r="A10" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5">
+      <c r="B10" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3">
         <v>13321</v>
       </c>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5" t="s">
+      <c r="H10" s="3"/>
+      <c r="I10" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J10" s="4"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5">
+      <c r="K10" s="3"/>
+      <c r="L10" s="3">
         <v>10638</v>
       </c>
-      <c r="M10" s="5"/>
-      <c r="N10" s="5">
+      <c r="M10" s="3"/>
+      <c r="N10" s="3">
         <v>13488</v>
       </c>
       <c r="O10" s="1"/>
@@ -694,27 +707,26 @@
       <c r="A11" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5">
+      <c r="B11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3">
         <v>14292</v>
       </c>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5">
+      <c r="H11" s="3"/>
+      <c r="I11" s="3">
         <v>8858</v>
       </c>
-      <c r="J11" s="4"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5">
+      <c r="K11" s="3"/>
+      <c r="L11" s="3">
         <v>10947</v>
       </c>
-      <c r="M11" s="5"/>
-      <c r="N11" s="5">
+      <c r="M11" s="3"/>
+      <c r="N11" s="3">
         <v>13788</v>
       </c>
       <c r="O11" s="1"/>
@@ -724,27 +736,26 @@
       <c r="A12" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5">
+      <c r="B12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3">
         <v>13816</v>
       </c>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5">
+      <c r="H12" s="3"/>
+      <c r="I12" s="3">
         <v>9058</v>
       </c>
-      <c r="J12" s="4"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5">
+      <c r="K12" s="3"/>
+      <c r="L12" s="3">
         <v>10806</v>
       </c>
-      <c r="M12" s="5"/>
-      <c r="N12" s="5"/>
+      <c r="M12" s="3"/>
+      <c r="N12" s="3"/>
       <c r="O12" s="1"/>
       <c r="P12" s="1"/>
     </row>
@@ -752,27 +763,26 @@
       <c r="A13" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="4">
-        <v>1</v>
-      </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5">
+      <c r="B13" s="2">
+        <v>1</v>
+      </c>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3">
         <v>9218</v>
       </c>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5">
+      <c r="H13" s="3"/>
+      <c r="I13" s="3">
         <v>8801</v>
       </c>
-      <c r="J13" s="4"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5">
+      <c r="K13" s="3"/>
+      <c r="L13" s="3">
         <v>10029</v>
       </c>
-      <c r="M13" s="5"/>
-      <c r="N13" s="5"/>
+      <c r="M13" s="3"/>
+      <c r="N13" s="3"/>
       <c r="O13" s="1"/>
       <c r="P13" s="1"/>
     </row>
@@ -780,25 +790,24 @@
       <c r="A14" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="4">
-        <v>1</v>
-      </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5">
+      <c r="B14" s="2">
+        <v>1</v>
+      </c>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3">
         <v>9483</v>
       </c>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5">
+      <c r="H14" s="3"/>
+      <c r="I14" s="3">
         <v>10494</v>
       </c>
-      <c r="J14" s="4"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
+      <c r="M14" s="3"/>
+      <c r="N14" s="3"/>
       <c r="O14" s="1"/>
       <c r="P14" s="1"/>
     </row>
@@ -806,117 +815,102 @@
       <c r="A15" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="4">
+      <c r="B15" s="2">
         <v>2</v>
       </c>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5">
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3">
         <v>2956</v>
       </c>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5">
+      <c r="I15" s="3"/>
+      <c r="J15" s="3">
         <v>2884</v>
       </c>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5" t="s">
+      <c r="K15" s="3"/>
+      <c r="L15" s="3"/>
+      <c r="M15" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="N15" s="5"/>
+      <c r="N15" s="3"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="4">
+      <c r="B16" s="2">
         <v>3</v>
       </c>
-      <c r="C16" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4" t="s">
+      <c r="C16" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H16" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4" t="s">
+      <c r="J16" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="K16" s="4"/>
-      <c r="L16" s="4"/>
-      <c r="M16" s="5">
+      <c r="M16" s="3">
         <v>3204</v>
       </c>
-      <c r="N16" s="5"/>
+      <c r="N16" s="3"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="4">
+      <c r="B17" s="2">
         <v>6</v>
       </c>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="5">
+      <c r="H17" s="3">
         <v>2954</v>
       </c>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5">
+      <c r="I17" s="3"/>
+      <c r="J17" s="3">
         <v>2889</v>
       </c>
-      <c r="K17" s="5"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5">
+      <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
+      <c r="M17" s="3">
         <v>3217</v>
       </c>
-      <c r="N17" s="5"/>
+      <c r="N17" s="3"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="4">
+      <c r="B18" s="2">
         <v>10</v>
       </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="5">
+      <c r="H18" s="3">
         <v>2967</v>
       </c>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5">
+      <c r="I18" s="3"/>
+      <c r="J18" s="3">
         <v>2896</v>
       </c>
-      <c r="K18" s="5"/>
-      <c r="L18" s="5"/>
-      <c r="M18" s="5">
+      <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
+      <c r="M18" s="3">
         <v>3242</v>
       </c>
-      <c r="N18" s="5"/>
+      <c r="N18" s="3"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="4">
+      <c r="B19" s="2">
         <v>100</v>
       </c>
       <c r="G19" s="2" t="s">
@@ -933,7 +927,7 @@
       <c r="A20" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="4">
+      <c r="B20" s="2">
         <v>200</v>
       </c>
       <c r="G20" s="3">
@@ -1066,4 +1060,1810 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D540E39C-50CC-4B88-9879-4A057440D1BD}">
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="9.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="10.7109375" style="5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="6">
+        <v>40</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="5">
+        <v>7.32416</v>
+      </c>
+      <c r="D2" s="5">
+        <v>7.7979599999999998</v>
+      </c>
+      <c r="E2" s="5">
+        <v>7.4445499999999996</v>
+      </c>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="6">
+        <v>40</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="5">
+        <v>8.3222299999999994</v>
+      </c>
+      <c r="D3" s="5">
+        <v>7.8686699999999998</v>
+      </c>
+      <c r="E3" s="5">
+        <v>8.10656</v>
+      </c>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="6">
+        <v>40</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="5">
+        <v>10.3141</v>
+      </c>
+      <c r="D4" s="5">
+        <v>9.1351999999999993</v>
+      </c>
+      <c r="E4" s="5">
+        <v>8.6441700000000008</v>
+      </c>
+      <c r="F4" s="2"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="6">
+        <v>20</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="5">
+        <v>9.4985999999999997</v>
+      </c>
+      <c r="D5" s="5">
+        <v>7.9767900000000003</v>
+      </c>
+      <c r="E5" s="5">
+        <v>7.0766400000000003</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="6">
+        <v>20</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="5">
+        <v>10.520799999999999</v>
+      </c>
+      <c r="D6" s="5">
+        <v>9.00685</v>
+      </c>
+      <c r="E6" s="5">
+        <v>8.7744199999999992</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="6">
+        <v>20</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="5">
+        <v>11.707800000000001</v>
+      </c>
+      <c r="D7" s="5">
+        <v>9.8977500000000003</v>
+      </c>
+      <c r="E7" s="5">
+        <v>10.9466</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="6">
+        <v>12</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="5">
+        <v>9.4514499999999995</v>
+      </c>
+      <c r="D8" s="5">
+        <v>6.3848000000000003</v>
+      </c>
+      <c r="E8" s="5">
+        <v>7.8076299999999996</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="6">
+        <v>12</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="5">
+        <v>10.527699999999999</v>
+      </c>
+      <c r="D9" s="5">
+        <v>6.4290399999999996</v>
+      </c>
+      <c r="E9" s="5">
+        <v>8.4249200000000002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="6">
+        <v>12</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="5">
+        <v>12.9442</v>
+      </c>
+      <c r="D10" s="5">
+        <v>6.7478400000000001</v>
+      </c>
+      <c r="E10" s="5">
+        <v>9.5620799999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="6">
+        <v>6</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="5">
+        <v>15.8126</v>
+      </c>
+      <c r="D11" s="5">
+        <v>10.3872</v>
+      </c>
+      <c r="E11" s="5">
+        <v>11.3177</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="6">
+        <v>6</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="5">
+        <v>16.860499999999998</v>
+      </c>
+      <c r="D12" s="5">
+        <v>11.3195</v>
+      </c>
+      <c r="E12" s="5">
+        <v>12.301399999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="6">
+        <v>6</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="5">
+        <v>17.1312</v>
+      </c>
+      <c r="D13" s="5">
+        <v>11.4901</v>
+      </c>
+      <c r="E13" s="5">
+        <v>12.5357</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="6">
+        <v>3</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="5">
+        <v>26.828900000000001</v>
+      </c>
+      <c r="D14" s="5">
+        <v>16.991900000000001</v>
+      </c>
+      <c r="E14" s="5">
+        <v>18.972000000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="6">
+        <v>3</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="5">
+        <v>28.250499999999999</v>
+      </c>
+      <c r="D15" s="5">
+        <v>16.991399999999999</v>
+      </c>
+      <c r="E15" s="5">
+        <v>19.5242</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="6">
+        <v>3</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="5">
+        <v>27.869700000000002</v>
+      </c>
+      <c r="D16" s="5">
+        <v>16.967400000000001</v>
+      </c>
+      <c r="E16" s="5">
+        <v>19.510100000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="6">
+        <v>1</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" s="5">
+        <v>38.643900000000002</v>
+      </c>
+      <c r="D17" s="5">
+        <v>39.148200000000003</v>
+      </c>
+      <c r="E17" s="5">
+        <v>38.0458</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="6">
+        <v>1</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="5">
+        <v>39.251600000000003</v>
+      </c>
+      <c r="D18" s="5">
+        <v>39.2318</v>
+      </c>
+      <c r="E18" s="5">
+        <v>38.9285</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="6">
+        <v>1</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" s="5">
+        <v>39.411000000000001</v>
+      </c>
+      <c r="D19" s="5">
+        <v>39.132399999999997</v>
+      </c>
+      <c r="E19" s="5">
+        <v>39.124600000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6222A662-89DE-4BA6-B52E-9092C4D81900}">
+  <dimension ref="A1:E85"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10" style="7" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11" style="7" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="7">
+        <v>37.068899999999999</v>
+      </c>
+      <c r="D2" s="7">
+        <v>38.787599999999998</v>
+      </c>
+      <c r="E2" s="7">
+        <v>37.039099999999998</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2">
+        <v>1</v>
+      </c>
+      <c r="C3" s="7">
+        <v>38.123399999999997</v>
+      </c>
+      <c r="D3" s="7">
+        <v>39.823900000000002</v>
+      </c>
+      <c r="E3" s="7">
+        <v>38.009799999999998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2">
+        <v>1</v>
+      </c>
+      <c r="C4" s="7">
+        <v>38.226599999999998</v>
+      </c>
+      <c r="D4" s="7">
+        <v>39.846899999999998</v>
+      </c>
+      <c r="E4" s="7">
+        <v>38.146099999999997</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2">
+        <v>5</v>
+      </c>
+      <c r="C5" s="7">
+        <v>38.326999999999998</v>
+      </c>
+      <c r="D5" s="7">
+        <v>39.915999999999997</v>
+      </c>
+      <c r="E5" s="7">
+        <v>38.161099999999998</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>1</v>
+      </c>
+      <c r="B6" s="2">
+        <v>5</v>
+      </c>
+      <c r="C6" s="7">
+        <v>38.454799999999999</v>
+      </c>
+      <c r="D6" s="7">
+        <v>39.766399999999997</v>
+      </c>
+      <c r="E6" s="7">
+        <v>38.364199999999997</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>1</v>
+      </c>
+      <c r="B7" s="2">
+        <v>5</v>
+      </c>
+      <c r="C7" s="7">
+        <v>38.399000000000001</v>
+      </c>
+      <c r="D7" s="7">
+        <v>39.659399999999998</v>
+      </c>
+      <c r="E7" s="7">
+        <v>38.3765</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>1</v>
+      </c>
+      <c r="B8" s="2">
+        <v>10</v>
+      </c>
+      <c r="C8" s="7">
+        <v>38.865400000000001</v>
+      </c>
+      <c r="D8" s="7">
+        <v>39.611600000000003</v>
+      </c>
+      <c r="E8" s="7">
+        <v>38.400700000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>1</v>
+      </c>
+      <c r="B9" s="2">
+        <v>10</v>
+      </c>
+      <c r="C9" s="7">
+        <v>38.7881</v>
+      </c>
+      <c r="D9" s="7">
+        <v>39.795200000000001</v>
+      </c>
+      <c r="E9" s="7">
+        <v>38.430500000000002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>1</v>
+      </c>
+      <c r="B10" s="2">
+        <v>10</v>
+      </c>
+      <c r="C10" s="7">
+        <v>39.789099999999998</v>
+      </c>
+      <c r="D10" s="7">
+        <v>39.594299999999997</v>
+      </c>
+      <c r="E10" s="7">
+        <v>38.6081</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <v>1</v>
+      </c>
+      <c r="B11" s="2">
+        <v>20</v>
+      </c>
+      <c r="C11" s="7">
+        <v>41.9011</v>
+      </c>
+      <c r="D11" s="7">
+        <v>39.944699999999997</v>
+      </c>
+      <c r="E11" s="7">
+        <v>38.592700000000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>1</v>
+      </c>
+      <c r="B12" s="2">
+        <v>20</v>
+      </c>
+      <c r="C12" s="7">
+        <v>40.976300000000002</v>
+      </c>
+      <c r="D12" s="7">
+        <v>39.6188</v>
+      </c>
+      <c r="E12" s="7">
+        <v>38.497999999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <v>1</v>
+      </c>
+      <c r="B13" s="2">
+        <v>20</v>
+      </c>
+      <c r="C13" s="7">
+        <v>40.995699999999999</v>
+      </c>
+      <c r="D13" s="7">
+        <v>39.397399999999998</v>
+      </c>
+      <c r="E13" s="7">
+        <v>38.536299999999997</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>1</v>
+      </c>
+      <c r="B14" s="2">
+        <v>35</v>
+      </c>
+      <c r="C14" s="7">
+        <v>40.413499999999999</v>
+      </c>
+      <c r="D14" s="7">
+        <v>39.299900000000001</v>
+      </c>
+      <c r="E14" s="7">
+        <v>38.545099999999998</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
+        <v>1</v>
+      </c>
+      <c r="B15" s="2">
+        <v>35</v>
+      </c>
+      <c r="C15" s="7">
+        <v>40.779499999999999</v>
+      </c>
+      <c r="D15" s="7">
+        <v>39.246499999999997</v>
+      </c>
+      <c r="E15" s="7">
+        <v>38.814300000000003</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <v>1</v>
+      </c>
+      <c r="B16" s="2">
+        <v>35</v>
+      </c>
+      <c r="C16" s="7">
+        <v>40.806199999999997</v>
+      </c>
+      <c r="D16" s="7">
+        <v>39.014899999999997</v>
+      </c>
+      <c r="E16" s="7">
+        <v>38.661099999999998</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <v>1</v>
+      </c>
+      <c r="B17" s="2">
+        <v>50</v>
+      </c>
+      <c r="C17" s="7">
+        <v>40.773800000000001</v>
+      </c>
+      <c r="D17" s="7">
+        <v>39.429600000000001</v>
+      </c>
+      <c r="E17" s="7">
+        <v>38.567700000000002</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
+        <v>1</v>
+      </c>
+      <c r="B18" s="2">
+        <v>50</v>
+      </c>
+      <c r="C18" s="7">
+        <v>40.931199999999997</v>
+      </c>
+      <c r="D18" s="7">
+        <v>41.481499999999997</v>
+      </c>
+      <c r="E18" s="7">
+        <v>38.685099999999998</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" s="2">
+        <v>1</v>
+      </c>
+      <c r="B19" s="2">
+        <v>50</v>
+      </c>
+      <c r="C19" s="7">
+        <v>41.484900000000003</v>
+      </c>
+      <c r="D19" s="7">
+        <v>44.3215</v>
+      </c>
+      <c r="E19" s="7">
+        <v>38.834800000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="2">
+        <v>1</v>
+      </c>
+      <c r="B20" s="2">
+        <v>100</v>
+      </c>
+      <c r="C20" s="7">
+        <v>42.342100000000002</v>
+      </c>
+      <c r="D20" s="7">
+        <v>42.773800000000001</v>
+      </c>
+      <c r="E20" s="7">
+        <v>38.777900000000002</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="2">
+        <v>1</v>
+      </c>
+      <c r="B21" s="2">
+        <v>100</v>
+      </c>
+      <c r="C21" s="7">
+        <v>43.262</v>
+      </c>
+      <c r="D21" s="7">
+        <v>39.898200000000003</v>
+      </c>
+      <c r="E21" s="7">
+        <v>38.820999999999998</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="2">
+        <v>1</v>
+      </c>
+      <c r="B22" s="2">
+        <v>100</v>
+      </c>
+      <c r="C22" s="7">
+        <v>42.450800000000001</v>
+      </c>
+      <c r="D22" s="7">
+        <v>39.578899999999997</v>
+      </c>
+      <c r="E22" s="7">
+        <v>38.533499999999997</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="2">
+        <v>1</v>
+      </c>
+      <c r="B23" s="2">
+        <v>200</v>
+      </c>
+      <c r="C23" s="7">
+        <v>41.569099999999999</v>
+      </c>
+      <c r="D23" s="7">
+        <v>39.741700000000002</v>
+      </c>
+      <c r="E23" s="7">
+        <v>38.654200000000003</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="2">
+        <v>1</v>
+      </c>
+      <c r="B24" s="2">
+        <v>200</v>
+      </c>
+      <c r="C24" s="7">
+        <v>42.395299999999999</v>
+      </c>
+      <c r="D24" s="7">
+        <v>39.779499999999999</v>
+      </c>
+      <c r="E24" s="7">
+        <v>38.578299999999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="2">
+        <v>1</v>
+      </c>
+      <c r="B25" s="2">
+        <v>200</v>
+      </c>
+      <c r="C25" s="7">
+        <v>42.091900000000003</v>
+      </c>
+      <c r="D25" s="7">
+        <v>39.315300000000001</v>
+      </c>
+      <c r="E25" s="7">
+        <v>38.5655</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="2">
+        <v>1</v>
+      </c>
+      <c r="B26" s="2">
+        <v>500</v>
+      </c>
+      <c r="C26" s="7">
+        <v>41.357399999999998</v>
+      </c>
+      <c r="D26" s="7">
+        <v>39.478900000000003</v>
+      </c>
+      <c r="E26" s="7">
+        <v>38.602600000000002</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="2">
+        <v>1</v>
+      </c>
+      <c r="B27" s="2">
+        <v>500</v>
+      </c>
+      <c r="C27" s="7">
+        <v>43.89</v>
+      </c>
+      <c r="D27" s="7">
+        <v>39.208300000000001</v>
+      </c>
+      <c r="E27" s="7">
+        <v>38.651899999999998</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="2">
+        <v>1</v>
+      </c>
+      <c r="B28" s="2">
+        <v>500</v>
+      </c>
+      <c r="C28" s="7">
+        <v>44.879300000000001</v>
+      </c>
+      <c r="D28" s="7">
+        <v>39.281399999999998</v>
+      </c>
+      <c r="E28" s="7">
+        <v>38.739100000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="2">
+        <v>1</v>
+      </c>
+      <c r="B29" s="2">
+        <v>1000</v>
+      </c>
+      <c r="C29" s="7">
+        <v>41.406599999999997</v>
+      </c>
+      <c r="D29" s="7">
+        <v>39.320300000000003</v>
+      </c>
+      <c r="E29" s="7">
+        <v>38.660899999999998</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="2">
+        <v>1</v>
+      </c>
+      <c r="B30" s="2">
+        <v>1000</v>
+      </c>
+      <c r="C30" s="7">
+        <v>41.193899999999999</v>
+      </c>
+      <c r="D30" s="7">
+        <v>39.2744</v>
+      </c>
+      <c r="E30" s="7">
+        <v>38.736600000000003</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="2">
+        <v>1</v>
+      </c>
+      <c r="B31" s="2">
+        <v>1000</v>
+      </c>
+      <c r="C31" s="7">
+        <v>43.115200000000002</v>
+      </c>
+      <c r="D31" s="7">
+        <v>38.942500000000003</v>
+      </c>
+      <c r="E31" s="7">
+        <v>38.516199999999998</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="2">
+        <v>1</v>
+      </c>
+      <c r="B32" s="2">
+        <v>2000</v>
+      </c>
+      <c r="C32" s="7">
+        <v>46.492600000000003</v>
+      </c>
+      <c r="D32" s="7">
+        <v>39.226700000000001</v>
+      </c>
+      <c r="E32" s="7">
+        <v>38.688600000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="2">
+        <v>1</v>
+      </c>
+      <c r="B33" s="2">
+        <v>2000</v>
+      </c>
+      <c r="C33" s="7">
+        <v>46.906700000000001</v>
+      </c>
+      <c r="D33" s="7">
+        <v>39.055100000000003</v>
+      </c>
+      <c r="E33" s="7">
+        <v>40.049799999999998</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="2">
+        <v>1</v>
+      </c>
+      <c r="B34" s="2">
+        <v>2000</v>
+      </c>
+      <c r="C34" s="7">
+        <v>45.492199999999997</v>
+      </c>
+      <c r="D34" s="7">
+        <v>39.174599999999998</v>
+      </c>
+      <c r="E34" s="7">
+        <v>40.416800000000002</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="2">
+        <v>1</v>
+      </c>
+      <c r="B35" s="2">
+        <v>4000</v>
+      </c>
+      <c r="C35" s="7">
+        <v>43.687899999999999</v>
+      </c>
+      <c r="D35" s="7">
+        <v>39.139400000000002</v>
+      </c>
+      <c r="E35" s="7">
+        <v>39.474200000000003</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="2">
+        <v>1</v>
+      </c>
+      <c r="B36" s="2">
+        <v>4000</v>
+      </c>
+      <c r="C36" s="7">
+        <v>44.584499999999998</v>
+      </c>
+      <c r="D36" s="7">
+        <v>39.2697</v>
+      </c>
+      <c r="E36" s="7">
+        <v>38.702100000000002</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="2">
+        <v>1</v>
+      </c>
+      <c r="B37" s="2">
+        <v>4000</v>
+      </c>
+      <c r="C37" s="7">
+        <v>44.180999999999997</v>
+      </c>
+      <c r="D37" s="7">
+        <v>39.058300000000003</v>
+      </c>
+      <c r="E37" s="7">
+        <v>38.85</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="2">
+        <v>1</v>
+      </c>
+      <c r="B38" s="2">
+        <v>8000</v>
+      </c>
+      <c r="C38" s="7">
+        <v>42.554499999999997</v>
+      </c>
+      <c r="D38" s="7">
+        <v>39.3752</v>
+      </c>
+      <c r="E38" s="7">
+        <v>38.763300000000001</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" s="2">
+        <v>1</v>
+      </c>
+      <c r="B39" s="2">
+        <v>8000</v>
+      </c>
+      <c r="C39" s="7">
+        <v>40.695500000000003</v>
+      </c>
+      <c r="D39" s="7">
+        <v>39.055500000000002</v>
+      </c>
+      <c r="E39" s="7">
+        <v>38.354300000000002</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="2">
+        <v>1</v>
+      </c>
+      <c r="B40" s="2">
+        <v>8000</v>
+      </c>
+      <c r="C40" s="7">
+        <v>41.864800000000002</v>
+      </c>
+      <c r="D40" s="7">
+        <v>38.984299999999998</v>
+      </c>
+      <c r="E40" s="7">
+        <v>38.557299999999998</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="2">
+        <v>1</v>
+      </c>
+      <c r="B41" s="2">
+        <v>16000</v>
+      </c>
+      <c r="C41" s="7">
+        <v>41.659799999999997</v>
+      </c>
+      <c r="D41" s="7">
+        <v>39.328200000000002</v>
+      </c>
+      <c r="E41" s="7">
+        <v>39.311199999999999</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="2">
+        <v>1</v>
+      </c>
+      <c r="B42" s="2">
+        <v>16000</v>
+      </c>
+      <c r="C42" s="7">
+        <v>41.551200000000001</v>
+      </c>
+      <c r="D42" s="7">
+        <v>39.488500000000002</v>
+      </c>
+      <c r="E42" s="7">
+        <v>40.011200000000002</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="2">
+        <v>1</v>
+      </c>
+      <c r="B43" s="2">
+        <v>16000</v>
+      </c>
+      <c r="C43" s="7">
+        <v>41.595399999999998</v>
+      </c>
+      <c r="D43" s="7">
+        <v>39.308900000000001</v>
+      </c>
+      <c r="E43" s="7">
+        <v>40.151000000000003</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="2">
+        <v>12</v>
+      </c>
+      <c r="B44" s="2">
+        <v>1</v>
+      </c>
+      <c r="C44" s="7">
+        <v>6.7430500000000002</v>
+      </c>
+      <c r="D44" s="7">
+        <v>6.62256</v>
+      </c>
+      <c r="E44" s="7">
+        <v>6.8482500000000002</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="2">
+        <v>12</v>
+      </c>
+      <c r="B45" s="2">
+        <v>1</v>
+      </c>
+      <c r="C45" s="7">
+        <v>7.0716299999999999</v>
+      </c>
+      <c r="D45" s="7">
+        <v>7.8140200000000002</v>
+      </c>
+      <c r="E45" s="7">
+        <v>7.4223299999999997</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" s="2">
+        <v>12</v>
+      </c>
+      <c r="B46" s="2">
+        <v>1</v>
+      </c>
+      <c r="C46" s="7">
+        <v>8.1244999999999994</v>
+      </c>
+      <c r="D46" s="7">
+        <v>7.8787900000000004</v>
+      </c>
+      <c r="E46" s="7">
+        <v>7.8297699999999999</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" s="2">
+        <v>12</v>
+      </c>
+      <c r="B47" s="2">
+        <v>5</v>
+      </c>
+      <c r="C47" s="7">
+        <v>8.5501699999999996</v>
+      </c>
+      <c r="D47" s="7">
+        <v>7.7694400000000003</v>
+      </c>
+      <c r="E47" s="7">
+        <v>8.09389</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" s="2">
+        <v>12</v>
+      </c>
+      <c r="B48" s="2">
+        <v>5</v>
+      </c>
+      <c r="C48" s="7">
+        <v>7.9116400000000002</v>
+      </c>
+      <c r="D48" s="7">
+        <v>7.4296499999999996</v>
+      </c>
+      <c r="E48" s="7">
+        <v>8.0577900000000007</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="2">
+        <v>12</v>
+      </c>
+      <c r="B49" s="2">
+        <v>5</v>
+      </c>
+      <c r="C49" s="7">
+        <v>7.65665</v>
+      </c>
+      <c r="D49" s="7">
+        <v>7.5704500000000001</v>
+      </c>
+      <c r="E49" s="7">
+        <v>8.0259</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="2">
+        <v>12</v>
+      </c>
+      <c r="B50" s="2">
+        <v>10</v>
+      </c>
+      <c r="C50" s="7">
+        <v>7.9410499999999997</v>
+      </c>
+      <c r="D50" s="7">
+        <v>7.7773399999999997</v>
+      </c>
+      <c r="E50" s="7">
+        <v>8.2893899999999991</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="2">
+        <v>12</v>
+      </c>
+      <c r="B51" s="2">
+        <v>10</v>
+      </c>
+      <c r="C51" s="7">
+        <v>8.5381499999999999</v>
+      </c>
+      <c r="D51" s="7">
+        <v>7.7416799999999997</v>
+      </c>
+      <c r="E51" s="7">
+        <v>7.899</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="2">
+        <v>12</v>
+      </c>
+      <c r="B52" s="2">
+        <v>10</v>
+      </c>
+      <c r="C52" s="7">
+        <v>8.2006099999999993</v>
+      </c>
+      <c r="D52" s="7">
+        <v>8.4931599999999996</v>
+      </c>
+      <c r="E52" s="7">
+        <v>7.7622799999999996</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="2">
+        <v>12</v>
+      </c>
+      <c r="B53" s="2">
+        <v>20</v>
+      </c>
+      <c r="C53" s="7">
+        <v>7.5266599999999997</v>
+      </c>
+      <c r="D53" s="7">
+        <v>7.2465099999999998</v>
+      </c>
+      <c r="E53" s="7">
+        <v>7.9923900000000003</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="2">
+        <v>12</v>
+      </c>
+      <c r="B54" s="2">
+        <v>20</v>
+      </c>
+      <c r="C54" s="7">
+        <v>8.1009200000000003</v>
+      </c>
+      <c r="D54" s="7">
+        <v>7.02996</v>
+      </c>
+      <c r="E54" s="7">
+        <v>8.4397500000000001</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" s="2">
+        <v>12</v>
+      </c>
+      <c r="B55" s="2">
+        <v>20</v>
+      </c>
+      <c r="C55" s="7">
+        <v>11.4305</v>
+      </c>
+      <c r="D55" s="7">
+        <v>6.9788300000000003</v>
+      </c>
+      <c r="E55" s="7">
+        <v>7.71591</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="2">
+        <v>12</v>
+      </c>
+      <c r="B56" s="2">
+        <v>35</v>
+      </c>
+      <c r="C56" s="7">
+        <v>8.0953900000000001</v>
+      </c>
+      <c r="D56" s="7">
+        <v>7.03179</v>
+      </c>
+      <c r="E56" s="7">
+        <v>8.4648199999999996</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" s="2">
+        <v>12</v>
+      </c>
+      <c r="B57" s="2">
+        <v>35</v>
+      </c>
+      <c r="C57" s="7">
+        <v>9.0491399999999995</v>
+      </c>
+      <c r="D57" s="7">
+        <v>7.0245199999999999</v>
+      </c>
+      <c r="E57" s="7">
+        <v>8.5402900000000006</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" s="2">
+        <v>12</v>
+      </c>
+      <c r="B58" s="2">
+        <v>35</v>
+      </c>
+      <c r="C58" s="7">
+        <v>8.2316599999999998</v>
+      </c>
+      <c r="D58" s="7">
+        <v>7.0192699999999997</v>
+      </c>
+      <c r="E58" s="7">
+        <v>8.1603399999999997</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="2">
+        <v>12</v>
+      </c>
+      <c r="B59" s="2">
+        <v>50</v>
+      </c>
+      <c r="C59" s="7">
+        <v>7.7545999999999999</v>
+      </c>
+      <c r="D59" s="7">
+        <v>6.9482400000000002</v>
+      </c>
+      <c r="E59" s="7">
+        <v>7.9911899999999996</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" s="2">
+        <v>12</v>
+      </c>
+      <c r="B60" s="2">
+        <v>50</v>
+      </c>
+      <c r="C60" s="7">
+        <v>8.0014199999999995</v>
+      </c>
+      <c r="D60" s="7">
+        <v>7.2474600000000002</v>
+      </c>
+      <c r="E60" s="7">
+        <v>8.0271699999999999</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" s="2">
+        <v>12</v>
+      </c>
+      <c r="B61" s="2">
+        <v>50</v>
+      </c>
+      <c r="C61" s="7">
+        <v>7.7604499999999996</v>
+      </c>
+      <c r="D61" s="7">
+        <v>7.7061200000000003</v>
+      </c>
+      <c r="E61" s="7">
+        <v>7.6904599999999999</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" s="2">
+        <v>12</v>
+      </c>
+      <c r="B62" s="2">
+        <v>100</v>
+      </c>
+      <c r="C62" s="7">
+        <v>7.9967899999999998</v>
+      </c>
+      <c r="D62" s="7">
+        <v>7.3240499999999997</v>
+      </c>
+      <c r="E62" s="7">
+        <v>7.8746299999999998</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" s="2">
+        <v>12</v>
+      </c>
+      <c r="B63" s="2">
+        <v>100</v>
+      </c>
+      <c r="C63" s="7">
+        <v>7.9498100000000003</v>
+      </c>
+      <c r="D63" s="7">
+        <v>7.3414200000000003</v>
+      </c>
+      <c r="E63" s="7">
+        <v>7.8661099999999999</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="2">
+        <v>12</v>
+      </c>
+      <c r="B64" s="2">
+        <v>100</v>
+      </c>
+      <c r="C64" s="7">
+        <v>7.6017999999999999</v>
+      </c>
+      <c r="D64" s="7">
+        <v>7.3986299999999998</v>
+      </c>
+      <c r="E64" s="7">
+        <v>7.9466599999999996</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="2">
+        <v>12</v>
+      </c>
+      <c r="B65" s="2">
+        <v>200</v>
+      </c>
+      <c r="C65" s="7">
+        <v>9.5023</v>
+      </c>
+      <c r="D65" s="7">
+        <v>8.6872299999999996</v>
+      </c>
+      <c r="E65" s="7">
+        <v>9.3204700000000003</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" s="2">
+        <v>12</v>
+      </c>
+      <c r="B66" s="2">
+        <v>200</v>
+      </c>
+      <c r="C66" s="7">
+        <v>9.7144200000000005</v>
+      </c>
+      <c r="D66" s="7">
+        <v>8.7587200000000003</v>
+      </c>
+      <c r="E66" s="7">
+        <v>11.127700000000001</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" s="2">
+        <v>12</v>
+      </c>
+      <c r="B67" s="2">
+        <v>200</v>
+      </c>
+      <c r="C67" s="7">
+        <v>9.3639100000000006</v>
+      </c>
+      <c r="D67" s="7">
+        <v>8.7598199999999995</v>
+      </c>
+      <c r="E67" s="7">
+        <v>12.754799999999999</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="2">
+        <v>12</v>
+      </c>
+      <c r="B68" s="2">
+        <v>500</v>
+      </c>
+      <c r="C68" s="7">
+        <v>17.1524</v>
+      </c>
+      <c r="D68" s="7">
+        <v>15.773099999999999</v>
+      </c>
+      <c r="E68" s="7">
+        <v>16.702100000000002</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" s="2">
+        <v>12</v>
+      </c>
+      <c r="B69" s="2">
+        <v>500</v>
+      </c>
+      <c r="C69" s="7">
+        <v>17.6736</v>
+      </c>
+      <c r="D69" s="7">
+        <v>15.6251</v>
+      </c>
+      <c r="E69" s="7">
+        <v>16.191099999999999</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" s="2">
+        <v>12</v>
+      </c>
+      <c r="B70" s="2">
+        <v>500</v>
+      </c>
+      <c r="C70" s="7">
+        <v>16.941700000000001</v>
+      </c>
+      <c r="D70" s="7">
+        <v>15.7806</v>
+      </c>
+      <c r="E70" s="7">
+        <v>16.0291</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" s="2">
+        <v>12</v>
+      </c>
+      <c r="B71" s="2">
+        <v>1000</v>
+      </c>
+      <c r="C71" s="7">
+        <v>25.9133</v>
+      </c>
+      <c r="D71" s="7">
+        <v>24.748000000000001</v>
+      </c>
+      <c r="E71" s="7">
+        <v>24.994800000000001</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" s="2">
+        <v>12</v>
+      </c>
+      <c r="B72" s="2">
+        <v>1000</v>
+      </c>
+      <c r="C72" s="7">
+        <v>26.978000000000002</v>
+      </c>
+      <c r="D72" s="7">
+        <v>24.5503</v>
+      </c>
+      <c r="E72" s="7">
+        <v>25.496300000000002</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" s="2">
+        <v>12</v>
+      </c>
+      <c r="B73" s="2">
+        <v>1000</v>
+      </c>
+      <c r="C73" s="7">
+        <v>25.442299999999999</v>
+      </c>
+      <c r="D73" s="7">
+        <v>24.454499999999999</v>
+      </c>
+      <c r="E73" s="7">
+        <v>24.738800000000001</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="2">
+        <v>12</v>
+      </c>
+      <c r="B74" s="2">
+        <v>2000</v>
+      </c>
+      <c r="C74" s="7">
+        <v>31.904</v>
+      </c>
+      <c r="D74" s="7">
+        <v>29.335100000000001</v>
+      </c>
+      <c r="E74" s="7">
+        <v>29.699300000000001</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="2">
+        <v>12</v>
+      </c>
+      <c r="B75" s="2">
+        <v>2000</v>
+      </c>
+      <c r="C75" s="7">
+        <v>31.251200000000001</v>
+      </c>
+      <c r="D75" s="7">
+        <v>29.127700000000001</v>
+      </c>
+      <c r="E75" s="7">
+        <v>29.0825</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" s="2">
+        <v>12</v>
+      </c>
+      <c r="B76" s="2">
+        <v>2000</v>
+      </c>
+      <c r="C76" s="7">
+        <v>29.8538</v>
+      </c>
+      <c r="D76" s="7">
+        <v>29.060500000000001</v>
+      </c>
+      <c r="E76" s="7">
+        <v>29.194800000000001</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" s="2">
+        <v>12</v>
+      </c>
+      <c r="B77" s="2">
+        <v>4000</v>
+      </c>
+      <c r="C77" s="7">
+        <v>40.714199999999998</v>
+      </c>
+      <c r="D77" s="7">
+        <v>39.306199999999997</v>
+      </c>
+      <c r="E77" s="7">
+        <v>39.187399999999997</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A78" s="2">
+        <v>12</v>
+      </c>
+      <c r="B78" s="2">
+        <v>4000</v>
+      </c>
+      <c r="C78" s="7">
+        <v>40.451000000000001</v>
+      </c>
+      <c r="D78" s="7">
+        <v>39.542400000000001</v>
+      </c>
+      <c r="E78" s="7">
+        <v>39.111499999999999</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" s="2">
+        <v>12</v>
+      </c>
+      <c r="B79" s="2">
+        <v>4000</v>
+      </c>
+      <c r="C79" s="7">
+        <v>40.188899999999997</v>
+      </c>
+      <c r="D79" s="7">
+        <v>39.305999999999997</v>
+      </c>
+      <c r="E79" s="7">
+        <v>38.9602</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" s="2">
+        <v>12</v>
+      </c>
+      <c r="B80" s="2">
+        <v>8000</v>
+      </c>
+      <c r="C80" s="7">
+        <v>40.260399999999997</v>
+      </c>
+      <c r="D80" s="7">
+        <v>40.344200000000001</v>
+      </c>
+      <c r="E80" s="7">
+        <v>38.911200000000001</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" s="2">
+        <v>12</v>
+      </c>
+      <c r="B81" s="2">
+        <v>8000</v>
+      </c>
+      <c r="C81" s="7">
+        <v>40.3489</v>
+      </c>
+      <c r="D81" s="7">
+        <v>42.226100000000002</v>
+      </c>
+      <c r="E81" s="7">
+        <v>39.176200000000001</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" s="2">
+        <v>12</v>
+      </c>
+      <c r="B82" s="2">
+        <v>8000</v>
+      </c>
+      <c r="C82" s="7">
+        <v>40.917999999999999</v>
+      </c>
+      <c r="D82" s="7">
+        <v>39.964399999999998</v>
+      </c>
+      <c r="E82" s="7">
+        <v>38.887099999999997</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="2">
+        <v>12</v>
+      </c>
+      <c r="B83" s="2">
+        <v>16000</v>
+      </c>
+      <c r="C83" s="7">
+        <v>40.395899999999997</v>
+      </c>
+      <c r="D83" s="7">
+        <v>39.962400000000002</v>
+      </c>
+      <c r="E83" s="7">
+        <v>38.982799999999997</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" s="2">
+        <v>12</v>
+      </c>
+      <c r="B84" s="2">
+        <v>16000</v>
+      </c>
+      <c r="C84" s="7">
+        <v>39.907299999999999</v>
+      </c>
+      <c r="D84" s="7">
+        <v>41.074399999999997</v>
+      </c>
+      <c r="E84" s="7">
+        <v>39.107799999999997</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A85" s="2">
+        <v>12</v>
+      </c>
+      <c r="B85" s="2">
+        <v>16000</v>
+      </c>
+      <c r="C85" s="7">
+        <v>39.880600000000001</v>
+      </c>
+      <c r="D85" s="7">
+        <v>39.866300000000003</v>
+      </c>
+      <c r="E85" s="7">
+        <v>38.497799999999998</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>